<commit_message>
Hoan thien bai nop voi case Klarna va baseline cong khai
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong quan" sheetId="1" r:id="R296d99230a9f4007"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chan doan" sheetId="2" r:id="R623a79dcf3474e3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="3" r:id="R45b73effb07b494b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap 30-60-90" sheetId="4" r:id="R25d7fc5588c5467e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="5" r:id="R7320a69ab1834b25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phan bien" sheetId="6" r:id="R91d8b653714c44e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong quan" sheetId="1" r:id="R386ece09da2a40fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chan doan" sheetId="2" r:id="R733d177f782049ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="3" r:id="R0ed0bf934a1a4bc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap 30-60-90" sheetId="4" r:id="R8e2f23930020445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="5" r:id="Rc4cd15bcef874d8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phan bien" sheetId="6" r:id="R281a50c8894a42da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,9 +19,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="0.0%"/>
+    <x:numFmt numFmtId="200" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -47,18 +47,17 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FF16324F"/>
+      <x:color rgb="FF173653"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="10"/>
-      <x:color rgb="FF24313D"/>
+      <x:color rgb="FF173653"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:sz val="10"/>
-      <x:color rgb="FF24313D"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -70,13 +69,7 @@
     <x:font>
       <x:b/>
       <x:sz val="12"/>
-      <x:color rgb="FF16324F"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FF16324F"/>
+      <x:color rgb="FF173653"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -89,7 +82,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF16324F"/>
+        <x:fgColor rgb="FF173653"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -99,7 +92,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF0F766E"/>
+        <x:fgColor rgb="FF0F7B70"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -170,32 +163,32 @@
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FF0F766E"/>
+        <x:color rgb="FF0F7B70"/>
       </x:left>
       <x:top style="thin">
-        <x:color rgb="FF0F766E"/>
+        <x:color rgb="FF0F7B70"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FF0F766E"/>
+        <x:color rgb="FF0F7B70"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:top style="thin">
-        <x:color rgb="FF0F766E"/>
+        <x:color rgb="FF0F7B70"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FF0F766E"/>
+        <x:color rgb="FF0F7B70"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:right style="thin">
-        <x:color rgb="FF0F766E"/>
+        <x:color rgb="FF0F7B70"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FF0F766E"/>
+        <x:color rgb="FF0F7B70"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FF0F766E"/>
+        <x:color rgb="FF0F7B70"/>
       </x:bottom>
     </x:border>
     <x:border>
@@ -220,7 +213,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="76">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -357,47 +350,33 @@
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="2">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -417,17 +396,6 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF24313D"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF4CE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -637,7 +605,7 @@
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
   </x:cols>
@@ -668,9 +636,9 @@
       <x:c r="I2" s="4"/>
       <x:c r="J2" s="4"/>
     </x:row>
-    <x:row r="3" ht="34" customHeight="1">
+    <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>Case lớp: Trợ lý AI tra cứu tài liệu nội bộ | Bản hoàn thiện sau kiểm tra chéo</x:v>
+        <x:v>Case thực tế công khai: Klarna AI Assistant trong chăm sóc khách hàng | Dữ liệu SEC/Klarna 2024–2025</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -696,12 +664,12 @@
       <x:c r="I5" s="11"/>
       <x:c r="J5" s="11"/>
     </x:row>
-    <x:row r="6" ht="30" customHeight="1">
+    <x:row r="6" ht="36" customHeight="1">
       <x:c r="A6" s="23" t="str">
         <x:v>Sản phẩm AI</x:v>
       </x:c>
       <x:c r="B6" s="24" t="str">
-        <x:v>Trợ lý AI tra cứu tài liệu nội bộ</x:v>
+        <x:v>Klarna AI Assistant trong ứng dụng Klarna</x:v>
       </x:c>
       <x:c r="C6" s="24"/>
       <x:c r="D6" s="24"/>
@@ -712,12 +680,12 @@
       <x:c r="I6" s="24"/>
       <x:c r="J6" s="24"/>
     </x:row>
-    <x:row r="7" ht="30" customHeight="1">
+    <x:row r="7" ht="36" customHeight="1">
       <x:c r="A7" s="25" t="str">
         <x:v>Người dùng chính</x:v>
       </x:c>
       <x:c r="B7" s="26" t="str">
-        <x:v>Nhân viên vận hành</x:v>
+        <x:v>Khách hàng Klarna cần hỗ trợ mua sắm, thanh toán, hoàn tiền hoặc đổi trả</x:v>
       </x:c>
       <x:c r="C7" s="26"/>
       <x:c r="D7" s="26"/>
@@ -728,12 +696,12 @@
       <x:c r="I7" s="26"/>
       <x:c r="J7" s="26"/>
     </x:row>
-    <x:row r="8" ht="30" customHeight="1">
+    <x:row r="8" ht="36" customHeight="1">
       <x:c r="A8" s="25" t="str">
-        <x:v>Quy trình</x:v>
+        <x:v>4 workflow</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>Tìm tài liệu; tóm tắt; kiểm chứng; sử dụng / báo lỗi</x:v>
+        <x:v>Tiếp nhận câu hỏi → AI phân loại → AI giải quyết → chuyển người/QA/phản hồi</x:v>
       </x:c>
       <x:c r="C8" s="26"/>
       <x:c r="D8" s="26"/>
@@ -744,12 +712,12 @@
       <x:c r="I8" s="26"/>
       <x:c r="J8" s="26"/>
     </x:row>
-    <x:row r="9" ht="30" customHeight="1">
+    <x:row r="9" ht="36" customHeight="1">
       <x:c r="A9" s="25" t="str">
-        <x:v>Vấn đề quan sát</x:v>
+        <x:v>Vấn đề đo được</x:v>
       </x:c>
       <x:c r="B9" s="26" t="str">
-        <x:v>Công cụ đã triển khai nhưng người dùng quay lại tìm file hoặc hỏi đồng nghiệp; câu trả lời thiếu nguồn và ngày cập nhật.</x:v>
+        <x:v>Usage và năng suất rất cao, nhưng có bằng chứng công khai về chất lượng thấp hơn ở một số dịch vụ AI; cần cân bằng AI với hỗ trợ con người.</x:v>
       </x:c>
       <x:c r="C9" s="26"/>
       <x:c r="D9" s="26"/>
@@ -762,7 +730,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="11" t="str">
-        <x:v>02  TÌNH TRẠNG &amp; QUYẾT ĐỊNH</x:v>
+        <x:v>02  QUYẾT ĐỊNH TỰ ĐỘNG TỪ METRIC</x:v>
       </x:c>
       <x:c r="B11" s="11"/>
       <x:c r="C11" s="11"/>
@@ -774,14 +742,14 @@
       <x:c r="I11" s="11"/>
       <x:c r="J11" s="11"/>
     </x:row>
-    <x:row r="12" ht="42" customHeight="1">
+    <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="35" t="str">
         <x:v>QUYẾT ĐỊNH</x:v>
       </x:c>
       <x:c r="B12" s="36"/>
       <x:c r="C12" s="36" t="str">
-        <x:f>IF(COUNTIF('Metrics'!$I$6:$I$11,"XẤU")&gt;0,"SỬA",IF(COUNTIF('Metrics'!$I$6:$I$11,"CHƯA ĐO")&gt;0,"SỬA — ĐO PILOT","TIẾP TỤC"))</x:f>
-        <x:v>SỬA — ĐO PILOT</x:v>
+        <x:f>IF(COUNTIF('Metrics'!$I$6:$I$11,"XẤU")&gt;0,"SỬA","TIẾP TỤC")</x:f>
+        <x:v>SỬA</x:v>
       </x:c>
       <x:c r="D12" s="36"/>
       <x:c r="E12" s="36"/>
@@ -790,7 +758,7 @@
       </x:c>
       <x:c r="G12" s="36"/>
       <x:c r="H12" s="36" t="str">
-        <x:v>Workflow chưa chính thức + kiến trúc tin cậy còn thiếu</x:v>
+        <x:v>Tối ưu quá mạnh theo chi phí/khối lượng + handoff người–AI cho ca phức tạp chưa đủ rõ</x:v>
       </x:c>
       <x:c r="I12" s="36"/>
       <x:c r="J12" s="37"/>
@@ -802,7 +770,7 @@
       <x:c r="B14" s="47"/>
       <x:c r="C14" s="47" t="n">
         <x:f>COUNTIF('Metrics'!$I$6:$I$11,"ĐẠT")</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D14" s="47"/>
       <x:c r="E14" s="47" t="str">
@@ -811,20 +779,20 @@
       <x:c r="F14" s="47"/>
       <x:c r="G14" s="47" t="n">
         <x:f>COUNTIF('Metrics'!$I$6:$I$11,"XẤU")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H14" s="47"/>
       <x:c r="I14" s="47" t="str">
-        <x:v>Chưa đo</x:v>
+        <x:v>Tổng</x:v>
       </x:c>
       <x:c r="J14" s="48" t="n">
-        <x:f>COUNTIF('Metrics'!$I$6:$I$11,"CHƯA ĐO")</x:f>
+        <x:f>COUNTA('Metrics'!$C$6:$C$11)</x:f>
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="11" t="str">
-        <x:v>03  ĐIỀU KIỆN RA QUYẾT ĐỊNH Ở NGÀY 90</x:v>
+        <x:v>03  QUY TẮC QUYẾT ĐỊNH</x:v>
       </x:c>
       <x:c r="B16" s="11"/>
       <x:c r="C16" s="11"/>
@@ -836,12 +804,12 @@
       <x:c r="I16" s="11"/>
       <x:c r="J16" s="11"/>
     </x:row>
-    <x:row r="17" ht="38" customHeight="1">
+    <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="23" t="str">
-        <x:v>TIẾP TỤC / MỞ RỘNG</x:v>
+        <x:v>TIẾP TỤC</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>Tất cả metric bắt buộc đạt; 0 sự cố quyền truy cập; owner vận hành và data owner đã nhận trách nhiệm</x:v>
+        <x:v>Metric năng suất, hành vi và chất lượng cùng đạt; ca rủi ro cao luôn có đường chuyển người; không có sự kiện chất lượng nghiêm trọng.</x:v>
       </x:c>
       <x:c r="C17" s="24"/>
       <x:c r="D17" s="24"/>
@@ -852,12 +820,12 @@
       <x:c r="I17" s="24"/>
       <x:c r="J17" s="24"/>
     </x:row>
-    <x:row r="18" ht="38" customHeight="1">
+    <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="25" t="str">
         <x:v>SỬA</x:v>
       </x:c>
       <x:c r="B18" s="26" t="str">
-        <x:v>Có metric chất lượng/hành vi dưới mục tiêu nhưng rủi ro còn kiểm soát được; quay lại sửa nguồn, handoff hoặc hướng dẫn tại workflow</x:v>
+        <x:v>Có lợi ích rõ nhưng ít nhất một quality/risk metric xấu: giữ AI cho ca thường, tăng human-in-the-loop cho ca phức tạp.</x:v>
       </x:c>
       <x:c r="C18" s="26"/>
       <x:c r="D18" s="26"/>
@@ -868,12 +836,12 @@
       <x:c r="I18" s="26"/>
       <x:c r="J18" s="26"/>
     </x:row>
-    <x:row r="19" ht="38" customHeight="1">
+    <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="25" t="str">
         <x:v>DỪNG</x:v>
       </x:c>
       <x:c r="B19" s="26" t="str">
-        <x:v>Có sự cố truy cập nghiêm trọng, không xác lập được nguồn đáng tin hoặc lợi ích workflow không xuất hiện sau hai vòng sửa</x:v>
+        <x:v>Dừng workflow nếu xảy ra lỗi nghiêm trọng về quyền, tài chính hoặc không thể tạo đường chuyển người an toàn sau hai vòng sửa.</x:v>
       </x:c>
       <x:c r="C19" s="26"/>
       <x:c r="D19" s="26"/>
@@ -884,12 +852,12 @@
       <x:c r="I19" s="26"/>
       <x:c r="J19" s="26"/>
     </x:row>
-    <x:row r="20" ht="38" customHeight="1">
+    <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="25" t="str">
         <x:v>BƯỚC TIẾP THEO</x:v>
       </x:c>
       <x:c r="B20" s="26" t="str">
-        <x:v>Pilot 20–30 nhân viên vận hành; đo baseline tuần 1; bật trích nguồn và QA mẫu trước khi xem xét mở rộng</x:v>
+        <x:v>Chuẩn hoá taxonomy ca phức tạp, SLA chuyển người, QA mẫu và dashboard chất lượng trước khi tiếp tục mở rộng.</x:v>
       </x:c>
       <x:c r="C20" s="26"/>
       <x:c r="D20" s="26"/>
@@ -932,14 +900,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -964,9 +932,9 @@
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
     </x:row>
-    <x:row r="3" ht="34" customHeight="1">
+    <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>Dùng framework đúng chỗ; phân biệt triệu chứng với nguyên nhân và chỉ ghi bằng chứng có thể kiểm tra.</x:v>
+        <x:v>Bằng chứng được lấy từ hồ sơ SEC/Klarna; framework dùng để giải thích nguyên nhân, không chỉ dán nhãn.</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -996,25 +964,25 @@
         <x:v>Trục</x:v>
       </x:c>
       <x:c r="C6" s="57" t="str">
-        <x:v>Câu hỏi</x:v>
+        <x:v>Nhận định</x:v>
       </x:c>
       <x:c r="D6" s="57" t="str">
-        <x:v>Nhận định</x:v>
+        <x:v>Mức</x:v>
       </x:c>
       <x:c r="E6" s="57" t="str">
-        <x:v>Mức</x:v>
+        <x:v>Framework</x:v>
       </x:c>
       <x:c r="F6" s="57" t="str">
-        <x:v>Framework</x:v>
+        <x:v>Bằng chứng thực tế</x:v>
       </x:c>
       <x:c r="G6" s="57" t="str">
-        <x:v>Bằng chứng</x:v>
+        <x:v>Nguồn</x:v>
       </x:c>
       <x:c r="H6" s="58" t="str">
-        <x:v>Hàm ý hành động</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="62" customHeight="1">
+        <x:v>Hàm ý</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="78" customHeight="1">
       <x:c r="A7" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -1022,25 +990,25 @@
         <x:v>Workflow</x:v>
       </x:c>
       <x:c r="C7" s="24" t="str">
-        <x:v>AI có nằm trong công việc thật không?</x:v>
+        <x:v>AI giải quyết phần lớn chat nhưng ca phức tạp cần lựa chọn gặp người thật và SLA chuyển tuyến.</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
-        <x:v>Chưa có bước chính thức, handoff và người chịu trách nhiệm cuối.</x:v>
+        <x:v>GỐC</x:v>
       </x:c>
       <x:c r="E7" s="24" t="str">
-        <x:v>GỐC</x:v>
+        <x:v>Mollick</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
-        <x:v>Mollick</x:v>
+        <x:v>SEC ghi Klarna tiếp tục cho mọi khách hàng lựa chọn đại diện con người.</x:v>
       </x:c>
       <x:c r="G7" s="24" t="str">
-        <x:v>[Brief case Lab] Người dùng quay lại tìm file hoặc hỏi đồng nghiệp thay vì dùng công cụ.</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000162828025034998/filename1.htm</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str">
-        <x:v>Thiết kế TO-BE và RACI tại từng bước.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="62" customHeight="1">
+        <x:v>Phân loại ca; AI làm ca thường; người giữ quyền ở ca phức tạp.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="78" customHeight="1">
       <x:c r="A8" s="26" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -1048,25 +1016,25 @@
         <x:v>Con người</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>Kẹt ở động lực, kiến thức hay khả năng?</x:v>
+        <x:v>Niềm tin bị ảnh hưởng khi chất lượng thấp hơn; training người dùng không giải quyết được.</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>Ngại tin vì không thấy nguồn; chưa biết khi nào dùng / không dùng.</x:v>
+        <x:v>LIÊN QUAN</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>LIÊN QUAN</x:v>
+        <x:v>ADKAR — Desire</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>ADKAR</x:v>
+        <x:v>SEC staff letter dẫn lời CEO về một số dịch vụ AI có chất lượng thấp hơn.</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>[Brief case Lab] Câu trả lời không kèm nguồn và ngày cập nhật nên người dùng không dám tin.</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000000000025005760/filename1.pdf</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str">
-        <x:v>Hướng dẫn tại workflow + hỗ trợ thực hành.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="62" customHeight="1">
+        <x:v>Tăng minh bạch và khả năng gặp người thật.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="78" customHeight="1">
       <x:c r="A9" s="26" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -1074,25 +1042,25 @@
         <x:v>Sẵn sàng</x:v>
       </x:c>
       <x:c r="C9" s="26" t="str">
-        <x:v>Dữ liệu, quyền và governance đã đủ chưa?</x:v>
+        <x:v>Direction và hạ tầng đạt; absorption cần cơ chế học từ lỗi và owner chất lượng.</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
-        <x:v>Nguồn thiếu data owner, lịch cập nhật và quy tắc quyền rõ ràng.</x:v>
+        <x:v>LIÊN QUAN</x:v>
       </x:c>
       <x:c r="E9" s="26" t="str">
-        <x:v>GỐC</x:v>
+        <x:v>Gartner-Lite</x:v>
       </x:c>
       <x:c r="F9" s="26" t="str">
-        <x:v>Gartner-Lite</x:v>
+        <x:v>31 triệu hội thoại và 80% chat cho thấy khả năng triển khai lớn.</x:v>
       </x:c>
       <x:c r="G9" s="26" t="str">
-        <x:v>[Brief case Lab + AS-IS v1] Khó xác định bản tài liệu mới nhất. [Chưa kiểm chứng] Thiếu data owner / lịch cập nhật / ACL — xác nhận ở tuần 1.</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000200329226000007/klar-20251231.htm</x:v>
       </x:c>
       <x:c r="H9" s="26" t="str">
-        <x:v>Khoá nguồn, data owner, lịch rà soát và ACL.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="62" customHeight="1">
+        <x:v>Không mở rộng chỉ dựa trên volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="78" customHeight="1">
       <x:c r="A10" s="26" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -1100,25 +1068,25 @@
         <x:v>Tin cậy</x:v>
       </x:c>
       <x:c r="C10" s="26" t="str">
-        <x:v>AI sai thì phát hiện và xử lý thế nào?</x:v>
+        <x:v>Chất lượng tổng hợp 'on-par' không đủ bảo đảm cho mọi phân khúc/ca rủi ro.</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
-        <x:v>Thiếu trích nguồn, QA mẫu, ngưỡng không chắc và chuyển người.</x:v>
+        <x:v>GỐC</x:v>
       </x:c>
       <x:c r="E10" s="26" t="str">
-        <x:v>GỐC</x:v>
+        <x:v>Kiến trúc tin cậy</x:v>
       </x:c>
       <x:c r="F10" s="26" t="str">
-        <x:v>Kiến trúc tin cậy</x:v>
+        <x:v>SEC ghi satisfaction ngang người nhưng staff letter đồng thời nêu tín hiệu lower quality.</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
-        <x:v>[Brief case Lab] Không có bước QA, ngưỡng "không chắc" hay đường chuyển SME khi AI trả lời sai.</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000200329226000007/klar-20251231.htm</x:v>
       </x:c>
       <x:c r="H10" s="26" t="str">
-        <x:v>Nguồn → trích nguồn → QA → chuyển người → phản hồi.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="62" customHeight="1">
+        <x:v>Theo dõi chất lượng theo loại ca; QA mẫu và escalation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="78" customHeight="1">
       <x:c r="A11" s="26" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -1126,27 +1094,27 @@
         <x:v>Đo lường</x:v>
       </x:c>
       <x:c r="C11" s="26" t="str">
-        <x:v>Đang đo activity hay giá trị?</x:v>
+        <x:v>Chi phí và tốc độ tốt nhưng cần quality gate/human-access metric.</x:v>
       </x:c>
       <x:c r="D11" s="26" t="str">
-        <x:v>Dashboard chỉ đếm login và số câu hỏi.</x:v>
+        <x:v>GỐC</x:v>
       </x:c>
       <x:c r="E11" s="26" t="str">
-        <x:v>LIÊN QUAN</x:v>
+        <x:v>5 tầng đo lường</x:v>
       </x:c>
       <x:c r="F11" s="26" t="str">
-        <x:v>5 tầng đo lường</x:v>
+        <x:v>2 phút so với 12 phút; giảm 25% câu hỏi lặp; 39 triệu USD tiết kiệm năm 2024.</x:v>
       </x:c>
       <x:c r="G11" s="26" t="str">
-        <x:v>[Dashboard v1, sheet "Metrics v1"] 4 chỉ số đều là activity hoặc tự khai: login, số câu hỏi, thời gian tự khai.</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000200329226000007/klar-20251231.htm</x:v>
       </x:c>
       <x:c r="H11" s="26" t="str">
-        <x:v>Đo chất lượng, thời gian, làm lại và kết quả workflow.</x:v>
+        <x:v>Giữ productivity metric nhưng quyết định bằng quality/risk.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="11" t="str">
-        <x:v>KẾT LUẬN GARTNER-LITE / ADKAR</x:v>
+        <x:v>KẾT LUẬN FRAMEWORK</x:v>
       </x:c>
       <x:c r="B13" s="11"/>
       <x:c r="C13" s="11"/>
@@ -1156,174 +1124,134 @@
       <x:c r="G13" s="11"/>
       <x:c r="H13" s="11"/>
     </x:row>
-    <x:row r="14" ht="42" customHeight="1">
+    <x:row r="14">
       <x:c r="A14" s="56" t="str">
+        <x:v>Framework</x:v>
+      </x:c>
+      <x:c r="B14" s="57" t="str">
+        <x:v>Kết quả</x:v>
+      </x:c>
+      <x:c r="C14" s="57" t="str">
+        <x:v>Điểm nghẽn</x:v>
+      </x:c>
+      <x:c r="D14" s="57" t="str">
+        <x:v>Can thiệp</x:v>
+      </x:c>
+      <x:c r="E14" s="57" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="F14" s="57" t="str">
+        <x:v>Dấu hiệu hoàn thành</x:v>
+      </x:c>
+      <x:c r="G14" s="57" t="str">
+        <x:v>Nguồn kiểm chứng</x:v>
+      </x:c>
+      <x:c r="H14" s="58" t="str">
+        <x:v>Quyết định</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="72" customHeight="1">
+      <x:c r="A15" s="24" t="str">
         <x:v>Gartner-Lite</x:v>
       </x:c>
-      <x:c r="B14" s="57" t="str">
-        <x:v>Nhận định</x:v>
-      </x:c>
-      <x:c r="C14" s="57" t="str">
-        <x:v>Kết quả</x:v>
-      </x:c>
-      <x:c r="D14" s="58" t="str">
-        <x:v>Quyết định</x:v>
-      </x:c>
-      <x:c r="E14" s="56" t="str">
+      <x:c r="B15" s="24" t="str">
+        <x:v>Direction/Readiness: ĐẠT; Absorption: CẦN SỬA</x:v>
+      </x:c>
+      <x:c r="C15" s="24" t="str">
+        <x:v>Governance chất lượng theo phân khúc</x:v>
+      </x:c>
+      <x:c r="D15" s="24" t="str">
+        <x:v>Quality gate + owner + vòng phản hồi</x:v>
+      </x:c>
+      <x:c r="E15" s="24" t="str">
+        <x:v>Giang Minh Phú</x:v>
+      </x:c>
+      <x:c r="F15" s="24" t="str">
+        <x:v>Dashboard có quality/risk metric, không chỉ volume</x:v>
+      </x:c>
+      <x:c r="G15" s="24" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000200329226000007/klar-20251231.htm</x:v>
+      </x:c>
+      <x:c r="H15" s="24" t="str">
+        <x:v>Pilot sửa</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="72" customHeight="1">
+      <x:c r="A16" s="26" t="str">
+        <x:v>Mollick</x:v>
+      </x:c>
+      <x:c r="B16" s="26" t="str">
+        <x:v>AI hỗ trợ/tự động ca thường; người giữ quyền ở ca phức tạp</x:v>
+      </x:c>
+      <x:c r="C16" s="26" t="str">
+        <x:v>Handoff chưa đủ nổi bật</x:v>
+      </x:c>
+      <x:c r="D16" s="26" t="str">
+        <x:v>SLA chuyển người + quyền quyết định cuối</x:v>
+      </x:c>
+      <x:c r="E16" s="26" t="str">
+        <x:v>Trần Thị Kiều Oanh</x:v>
+      </x:c>
+      <x:c r="F16" s="26" t="str">
+        <x:v>100% ca phức tạp có đường chuyển người</x:v>
+      </x:c>
+      <x:c r="G16" s="26" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000162828025034998/filename1.htm</x:v>
+      </x:c>
+      <x:c r="H16" s="26" t="str">
+        <x:v>Thiết kế lại</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="72" customHeight="1">
+      <x:c r="A17" s="26" t="str">
         <x:v>ADKAR</x:v>
       </x:c>
-      <x:c r="F14" s="57" t="str">
-        <x:v>Trạng thái</x:v>
-      </x:c>
-      <x:c r="G14" s="57" t="str">
-        <x:v>Can thiệp</x:v>
-      </x:c>
-      <x:c r="H14" s="58" t="str">
-        <x:v>Chỉ báo</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="42" customHeight="1">
-      <x:c r="A15" s="24" t="str">
-        <x:v>Direction</x:v>
-      </x:c>
-      <x:c r="B15" s="24" t="str">
-        <x:v>Mục tiêu và nhóm người dùng đã rõ.</x:v>
-      </x:c>
-      <x:c r="C15" s="24" t="str">
-        <x:v>ĐẠT</x:v>
-      </x:c>
-      <x:c r="D15" s="24" t="str">
-        <x:v>Giữ phạm vi pilot hẹp.</x:v>
-      </x:c>
-      <x:c r="E15" s="24" t="str">
-        <x:v>Awareness</x:v>
-      </x:c>
-      <x:c r="F15" s="24" t="str">
-        <x:v>NGHẼN</x:v>
-      </x:c>
-      <x:c r="G15" s="24" t="str">
-        <x:v>Định nghĩa loại câu hỏi nên / không nên dùng AI.</x:v>
-      </x:c>
-      <x:c r="H15" s="24" t="str">
-        <x:v>Tỷ lệ chọn đúng workflow</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="42" customHeight="1">
-      <x:c r="A16" s="26" t="str">
-        <x:v>Readiness</x:v>
-      </x:c>
-      <x:c r="B16" s="26" t="str">
-        <x:v>Data owner, lịch cập nhật, ACL và governance chưa đủ.</x:v>
-      </x:c>
-      <x:c r="C16" s="26" t="str">
-        <x:v>THIẾU</x:v>
-      </x:c>
-      <x:c r="D16" s="26" t="str">
-        <x:v>Chưa rollout rộng.</x:v>
-      </x:c>
-      <x:c r="E16" s="26" t="str">
-        <x:v>Desire</x:v>
-      </x:c>
-      <x:c r="F16" s="26" t="str">
-        <x:v>NGHẼN</x:v>
-      </x:c>
-      <x:c r="G16" s="26" t="str">
-        <x:v>Hiển thị nguồn và ngày cập nhật.</x:v>
-      </x:c>
-      <x:c r="H16" s="26" t="str">
-        <x:v>Tỷ lệ quay lại theo workflow</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="42" customHeight="1">
-      <x:c r="A17" s="26" t="str">
-        <x:v>Absorption</x:v>
-      </x:c>
       <x:c r="B17" s="26" t="str">
-        <x:v>Chưa có owner chất lượng và vòng phản hồi lỗi.</x:v>
+        <x:v>Nghẽn chính: Desire</x:v>
       </x:c>
       <x:c r="C17" s="26" t="str">
-        <x:v>THIẾU</x:v>
+        <x:v>Niềm tin vào chất lượng/human option</x:v>
       </x:c>
       <x:c r="D17" s="26" t="str">
-        <x:v>Bổ sung vận hành trước scale.</x:v>
+        <x:v>Hiển thị tùy chọn gặp người; phản hồi rõ</x:v>
       </x:c>
       <x:c r="E17" s="26" t="str">
-        <x:v>Knowledge</x:v>
+        <x:v>Lê Thị Thuý</x:v>
       </x:c>
       <x:c r="F17" s="26" t="str">
-        <x:v>CẦN LÀM</x:v>
+        <x:v>Giảm khiếu nại chất lượng; tăng first-contact resolution</x:v>
       </x:c>
       <x:c r="G17" s="26" t="str">
-        <x:v>Checklist hỏi và kiểm chứng.</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000000000025005760/filename1.pdf</x:v>
       </x:c>
       <x:c r="H17" s="26" t="str">
-        <x:v>Tỷ lệ kiểm nguồn</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="42" customHeight="1">
+        <x:v>Không chỉ đào tạo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="72" customHeight="1">
       <x:c r="A18" s="26" t="str">
         <x:v>Kết luận</x:v>
       </x:c>
       <x:c r="B18" s="26" t="str">
-        <x:v>Pilot nhỏ để sửa readiness và absorption.</x:v>
+        <x:v>SỬA, không dừng</x:v>
       </x:c>
       <x:c r="C18" s="26" t="str">
+        <x:v>Lợi ích đã chứng minh nhưng có quality signal xấu</x:v>
+      </x:c>
+      <x:c r="D18" s="26" t="str">
+        <x:v>Cân bằng automation với human-in-the-loop</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="str">
+        <x:v>Cả nhóm</x:v>
+      </x:c>
+      <x:c r="F18" s="26" t="str">
+        <x:v>Quality gate đạt trước scale</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000162828025052805/exhibit992klarnapresenta.htm</x:v>
+      </x:c>
+      <x:c r="H18" s="26" t="str">
         <x:v>SỬA</x:v>
-      </x:c>
-      <x:c r="D18" s="26" t="str">
-        <x:v>Đánh giá lại tại gate ngày 60.</x:v>
-      </x:c>
-      <x:c r="E18" s="26" t="str">
-        <x:v>Ability</x:v>
-      </x:c>
-      <x:c r="F18" s="26" t="str">
-        <x:v>CẦN LÀM</x:v>
-      </x:c>
-      <x:c r="G18" s="26" t="str">
-        <x:v>Office hour + champion trong pilot.</x:v>
-      </x:c>
-      <x:c r="H18" s="26" t="str">
-        <x:v>Tỷ lệ hoàn thành không cần làm lại</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="42" customHeight="1">
-      <x:c r="A19" s="26" t="str">
-        <x:v>Nguồn tham khảo</x:v>
-      </x:c>
-      <x:c r="B19" s="26" t="str">
-        <x:v>NIST AI RMF: https://airc.nist.gov/RMF — bằng chứng hiện có là brief case Lab + dashboard v1; số định lượng đo ở tuần 1 pilot.</x:v>
-      </x:c>
-      <x:c r="C19" s="26" t="str">
-        <x:v>Case tham khảo</x:v>
-      </x:c>
-      <x:c r="D19" s="26" t="str">
-        <x:v>Morgan Stanley — bài học: độ tin cậy và đánh giá đi trước mở rộng.</x:v>
-      </x:c>
-      <x:c r="E19" s="26" t="str">
-        <x:v>Reinforcement</x:v>
-      </x:c>
-      <x:c r="F19" s="26" t="str">
-        <x:v>CẦN LÀM</x:v>
-      </x:c>
-      <x:c r="G19" s="26" t="str">
-        <x:v>Phản hồi lỗi + review hàng tuần.</x:v>
-      </x:c>
-      <x:c r="H19" s="26" t="str">
-        <x:v>Tỷ lệ lỗi lặp lại</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="42" customHeight="1">
-      <x:c r="E20" s="26" t="str">
-        <x:v>Kết luận</x:v>
-      </x:c>
-      <x:c r="F20" s="26" t="str">
-        <x:v>Training không đủ</x:v>
-      </x:c>
-      <x:c r="G20" s="26" t="str">
-        <x:v>Sửa tin cậy và workflow trước.</x:v>
-      </x:c>
-      <x:c r="H20" s="26" t="str">
-        <x:v>Đo hành vi + chất lượng</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1341,15 +1269,15 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -1376,9 +1304,9 @@
       <x:c r="H2" s="4"/>
       <x:c r="I2" s="4"/>
     </x:row>
-    <x:row r="3" ht="34" customHeight="1">
+    <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>Ba thay đổi bắt buộc: nguồn kiểm chứng · người chịu trách nhiệm · xử lý khi AI không chắc chắn.</x:v>
+        <x:v>AS-IS và TO-BE cùng một đơn vị so sánh: quy trình xử lý một yêu cầu hỗ trợ của khách hàng Klarna.</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -1391,13 +1319,13 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="11" t="str">
-        <x:v>AS-IS</x:v>
+        <x:v>AS-IS — TỐI ƯU VOLUME</x:v>
       </x:c>
       <x:c r="B5" s="11"/>
       <x:c r="C5" s="11"/>
       <x:c r="D5" s="11"/>
       <x:c r="F5" s="61" t="str">
-        <x:v>TO-BE</x:v>
+        <x:v>TO-BE — AI + HUMAN-IN-THE-LOOP</x:v>
       </x:c>
       <x:c r="G5" s="61"/>
       <x:c r="H5" s="61"/>
@@ -1411,7 +1339,7 @@
         <x:v>Thực hiện</x:v>
       </x:c>
       <x:c r="C6" s="57" t="str">
-        <x:v>Điểm đau</x:v>
+        <x:v>Rủi ro</x:v>
       </x:c>
       <x:c r="D6" s="58" t="str">
         <x:v>Owner</x:v>
@@ -1423,142 +1351,168 @@
         <x:v>Thực hiện</x:v>
       </x:c>
       <x:c r="H6" s="57" t="str">
-        <x:v>Kiểm soát / handoff</x:v>
+        <x:v>Kiểm soát/handoff</x:v>
       </x:c>
       <x:c r="I6" s="58" t="str">
         <x:v>RACI / Owner</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="46" customHeight="1">
+    <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>Tìm file ở nhiều thư mục</x:v>
+        <x:v>Khách hàng gửi yêu cầu</x:v>
       </x:c>
       <x:c r="C7" s="24" t="str">
-        <x:v>Mất thời gian; khó biết bản mới nhất</x:v>
+        <x:v>Chưa gắn mức độ phức tạp</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
-        <x:v>Nhân viên</x:v>
+        <x:v>Customer Service Ops</x:v>
       </x:c>
       <x:c r="F7" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="24" t="str">
-        <x:v>Đặt câu hỏi theo mẫu</x:v>
+        <x:v>Tiếp nhận + consent</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str">
-        <x:v>Chỉ dùng cho phạm vi đã công bố</x:v>
+        <x:v>Cho chọn AI hoặc người ngay từ đầu</x:v>
       </x:c>
       <x:c r="I7" s="24" t="str">
-        <x:v>Nhân viên vận hành (R)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="46" customHeight="1">
+        <x:v>Customer Service Ops (R)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="26" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>Hỏi đồng nghiệp</x:v>
+        <x:v>AI tiếp nhận và phân loại</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>Phụ thuộc kinh nghiệm cá nhân</x:v>
+        <x:v>Có thể phân loại sai ca nhạy cảm</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>Không rõ</x:v>
+        <x:v>AI Product</x:v>
       </x:c>
       <x:c r="F8" s="26" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>AI tìm và tóm tắt</x:v>
+        <x:v>Phân loại mức rủi ro</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str">
-        <x:v>Chỉ truy xuất nguồn đã duyệt</x:v>
+        <x:v>Luật rõ: tài chính, ID theft, khiếu nại → người</x:v>
       </x:c>
       <x:c r="I8" s="26" t="str">
-        <x:v>AI hỗ trợ</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="46" customHeight="1">
+        <x:v>Giang Minh Phú (A)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="26" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B9" s="26" t="str">
-        <x:v>Đọc và tự tóm tắt</x:v>
+        <x:v>AI tự giải quyết</x:v>
       </x:c>
       <x:c r="C9" s="26" t="str">
-        <x:v>Không nhất quán</x:v>
+        <x:v>Tối ưu tốc độ/chi phí có thể lấn chất lượng</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
-        <x:v>Nhân viên</x:v>
+        <x:v>AI Product</x:v>
       </x:c>
       <x:c r="F9" s="26" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="G9" s="26" t="str">
-        <x:v>Xem nguồn + ngày cập nhật</x:v>
+        <x:v>AI xử lý ca thường</x:v>
       </x:c>
       <x:c r="H9" s="26" t="str">
-        <x:v>Bắt buộc mở tối thiểu 1 nguồn</x:v>
+        <x:v>Guardrail + nguồn chính sách + audit log</x:v>
       </x:c>
       <x:c r="I9" s="26" t="str">
-        <x:v>Nhân viên vận hành (R)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="46" customHeight="1">
+        <x:v>AI hỗ trợ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="26" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B10" s="26" t="str">
-        <x:v>Dùng kết quả</x:v>
+        <x:v>Khách hàng hỏi lại nếu chưa ổn</x:v>
       </x:c>
       <x:c r="C10" s="26" t="str">
-        <x:v>Thiếu dấu vết kiểm chứng</x:v>
+        <x:v>Repeat inquiry là tín hiệu trễ</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
-        <x:v>Không rõ</x:v>
+        <x:v>Customer Service Ops</x:v>
       </x:c>
       <x:c r="F10" s="26" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
-        <x:v>Kiểm chứng nội dung</x:v>
+        <x:v>Kiểm tra confidence/intent</x:v>
       </x:c>
       <x:c r="H10" s="26" t="str">
-        <x:v>Ngoại lệ/rủi ro cao chuyển SME</x:v>
+        <x:v>Dưới ngưỡng hoặc hỏi lại lần 2 → chuyển người</x:v>
       </x:c>
       <x:c r="I10" s="26" t="str">
-        <x:v>SME / quản lý (A)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="46" customHeight="1">
+        <x:v>Lê Thị Thuý (R — QA)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="48" customHeight="1">
+      <x:c r="A11" s="26" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B11" s="26" t="str">
+        <x:v>Chuyển người khi cần</x:v>
+      </x:c>
+      <x:c r="C11" s="26" t="str">
+        <x:v>Lựa chọn/SLA chưa được đo như quality gate</x:v>
+      </x:c>
+      <x:c r="D11" s="26" t="str">
+        <x:v>Human Support</x:v>
+      </x:c>
       <x:c r="F11" s="26" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="G11" s="26" t="str">
-        <x:v>Dùng hoặc không dùng</x:v>
+        <x:v>Người xử lý ca phức tạp</x:v>
       </x:c>
       <x:c r="H11" s="26" t="str">
-        <x:v>Con người giữ quyền quyết định cuối</x:v>
+        <x:v>Con người giữ quyền quyết định và ngoại lệ</x:v>
       </x:c>
       <x:c r="I11" s="26" t="str">
-        <x:v>Chủ quy trình (A) — Trần Thị Kiều Oanh</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="46" customHeight="1">
+        <x:v>Trần Thị Kiều Oanh (A)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="48" customHeight="1">
       <x:c r="F12" s="26" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="G12" s="26" t="str">
-        <x:v>Báo lỗi và học lại</x:v>
+        <x:v>QA mẫu + phản hồi</x:v>
       </x:c>
       <x:c r="H12" s="26" t="str">
-        <x:v>Ticket có loại lỗi, nguồn, mức độ</x:v>
+        <x:v>Phân tầng theo loại ca, severity và root cause</x:v>
       </x:c>
       <x:c r="I12" s="26" t="str">
-        <x:v>AI Product Owner (R) — Giang Minh Phú</x:v>
+        <x:v>Lê Thị Thuý (R)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="48" customHeight="1">
+      <x:c r="F13" s="26" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G13" s="26" t="str">
+        <x:v>Cập nhật dashboard</x:v>
+      </x:c>
+      <x:c r="H13" s="26" t="str">
+        <x:v>Quality/risk quyết định scale, không chỉ cost</x:v>
+      </x:c>
+      <x:c r="I13" s="26" t="str">
+        <x:v>Giang Minh Phú (R)</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1585,7 +1539,7 @@
         <x:v>Điều kiện</x:v>
       </x:c>
       <x:c r="D15" s="57" t="str">
-        <x:v>Quyền quyết định</x:v>
+        <x:v>Quyền cuối</x:v>
       </x:c>
       <x:c r="E15" s="57" t="str">
         <x:v>Kiểm chứng</x:v>
@@ -1603,88 +1557,88 @@
         <x:v>Rủi ro</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="55" customHeight="1">
+    <x:row r="16" ht="62" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:v>Người giữ quyền</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
-        <x:v>Phê duyệt cuối, ngoại lệ, rủi ro</x:v>
+        <x:v>Ca tài chính/ID theft/khiếu nại/ngoại lệ</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>Luôn luôn</x:v>
+        <x:v>Luôn chuyển người</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
         <x:v>Con người</x:v>
       </x:c>
       <x:c r="E16" s="24" t="str">
-        <x:v>SME / quản lý</x:v>
+        <x:v>QA + policy</x:v>
       </x:c>
       <x:c r="F16" s="24" t="str">
-        <x:v>Không sử dụng kết quả; chuyển SME</x:v>
+        <x:v>Không dùng quyết định AI</x:v>
       </x:c>
       <x:c r="G16" s="24" t="str">
-        <x:v>Chủ quy trình (Trần Thị Kiều Oanh)</x:v>
+        <x:v>Trần Thị Kiều Oanh</x:v>
       </x:c>
       <x:c r="H16" s="24" t="str">
-        <x:v>Quyết định + ngoại lệ</x:v>
+        <x:v>Escalation log</x:v>
       </x:c>
       <x:c r="I16" s="24" t="str">
         <x:v>Cao</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="55" customHeight="1">
+    <x:row r="17" ht="62" customHeight="1">
       <x:c r="A17" s="26" t="str">
         <x:v>AI hỗ trợ</x:v>
       </x:c>
       <x:c r="B17" s="26" t="str">
-        <x:v>Tìm, tóm tắt, đề xuất nguồn</x:v>
+        <x:v>Tóm tắt lịch sử, đề xuất câu trả lời</x:v>
       </x:c>
       <x:c r="C17" s="26" t="str">
-        <x:v>Nguồn đã duyệt</x:v>
+        <x:v>Ca phức tạp đã chuyển</x:v>
       </x:c>
       <x:c r="D17" s="26" t="str">
         <x:v>Con người</x:v>
       </x:c>
       <x:c r="E17" s="26" t="str">
-        <x:v>Mở nguồn + đối chiếu</x:v>
+        <x:v>Agent kiểm trước gửi</x:v>
       </x:c>
       <x:c r="F17" s="26" t="str">
-        <x:v>Hiển thị không chắc; yêu cầu làm rõ</x:v>
+        <x:v>Hiển thị uncertainty</x:v>
       </x:c>
       <x:c r="G17" s="26" t="str">
-        <x:v>AI Product Owner (Giang Minh Phú)</x:v>
+        <x:v>Giang Minh Phú</x:v>
       </x:c>
       <x:c r="H17" s="26" t="str">
-        <x:v>Prompt + nguồn + feedback</x:v>
+        <x:v>Prompt/source log</x:v>
       </x:c>
       <x:c r="I17" s="26" t="str">
         <x:v>Vừa</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="55" customHeight="1">
+    <x:row r="18" ht="62" customHeight="1">
       <x:c r="A18" s="26" t="str">
         <x:v>AI tự động có kiểm soát</x:v>
       </x:c>
       <x:c r="B18" s="26" t="str">
-        <x:v>Gắn nhãn ticket phản hồi</x:v>
+        <x:v>FAQ, trạng thái, thao tác lặp lại</x:v>
       </x:c>
       <x:c r="C18" s="26" t="str">
-        <x:v>Tác vụ lặp lại, rủi ro thấp</x:v>
+        <x:v>Rủi ro thấp + confidence đạt</x:v>
       </x:c>
       <x:c r="D18" s="26" t="str">
-        <x:v>Quy tắc đã duyệt</x:v>
+        <x:v>Quy tắc duyệt</x:v>
       </x:c>
       <x:c r="E18" s="26" t="str">
-        <x:v>QA mẫu 10%</x:v>
+        <x:v>QA mẫu phân tầng</x:v>
       </x:c>
       <x:c r="F18" s="26" t="str">
-        <x:v>Chuyển hàng đợi thủ công</x:v>
+        <x:v>Chuyển người tự động</x:v>
       </x:c>
       <x:c r="G18" s="26" t="str">
-        <x:v>QA Lead (Lê Thị Thuý)</x:v>
+        <x:v>Lê Thị Thuý</x:v>
       </x:c>
       <x:c r="H18" s="26" t="str">
-        <x:v>Ticket log</x:v>
+        <x:v>QA/feedback log</x:v>
       </x:c>
       <x:c r="I18" s="26" t="str">
         <x:v>Thấp</x:v>
@@ -1707,11 +1661,11 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
   </x:cols>
@@ -1738,9 +1692,9 @@
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
     </x:row>
-    <x:row r="3" ht="34" customHeight="1">
+    <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>Mỗi giai đoạn là một cổng quyết định dựa trên bằng chứng, không tự động chuyển khi hết ngày.</x:v>
+        <x:v>Ba cổng quyết định dựa trên bằng chứng; owner là thành viên chịu trách nhiệm hoàn thiện thiết kế trong bài.</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -1776,79 +1730,79 @@
         <x:v>Trạng thái</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="100" customHeight="1">
+    <x:row r="6" ht="96" customHeight="1">
       <x:c r="A6" s="24" t="str">
         <x:v>0–30 ngày</x:v>
       </x:c>
       <x:c r="B6" s="24" t="str">
-        <x:v>Chứng minh vấn đề và khả năng đo</x:v>
+        <x:v>Khoá phạm vi và quality baseline</x:v>
       </x:c>
       <x:c r="C6" s="24" t="str">
-        <x:v>Khoá 4 workflow; lập danh mục nguồn; chỉ định data owner; đo baseline tuần 1; pilot 20–30 người.</x:v>
+        <x:v>Chuẩn hoá 4 workflow; taxonomy ca phức tạp; data dictionary; baseline từ SEC và log mẫu.</x:v>
       </x:c>
       <x:c r="D6" s="24" t="str">
-        <x:v>AI Product Owner (Giang Minh Phú)</x:v>
+        <x:v>Giang Minh Phú</x:v>
       </x:c>
       <x:c r="E6" s="24" t="str">
-        <x:v>AS-IS/TO-BE; data dictionary; baseline có log; danh sách nguồn + ACL</x:v>
+        <x:v>Danh mục metric + nguồn + RACI + baseline</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
-        <x:v>100% nguồn pilot có owner; thu được ≥80% trường dữ liệu metric; không có nguồn ngoài ACL</x:v>
+        <x:v>100% metric có baseline/target/source/owner; taxonomy được duyệt</x:v>
       </x:c>
       <x:c r="G6" s="24" t="str">
-        <x:v>Thu hẹp nguồn/workflow; sửa instrument; chưa qua ngày 31</x:v>
+        <x:v>Thu hẹp workflow; bổ sung định nghĩa dữ liệu</x:v>
       </x:c>
       <x:c r="H6" s="62" t="str">
-        <x:v>CHƯA BẮT ĐẦU</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="100" customHeight="1">
+        <x:v>ĐẠT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="96" customHeight="1">
       <x:c r="A7" s="26" t="str">
         <x:v>31–60 ngày</x:v>
       </x:c>
       <x:c r="B7" s="26" t="str">
-        <x:v>Chứng minh chất lượng và hành vi</x:v>
+        <x:v>Chứng minh handoff và chất lượng</x:v>
       </x:c>
       <x:c r="C7" s="26" t="str">
-        <x:v>Bật trích nguồn + ngày; QA mẫu 10%; checklist kiểm chứng; office hour; review lỗi hằng tuần.</x:v>
+        <x:v>Thiết kế SLA chuyển người; QA mẫu phân tầng; đo human-access và lỗi nghiêm trọng.</x:v>
       </x:c>
       <x:c r="D7" s="26" t="str">
-        <x:v>QA Lead (Lê Thị Thuý)</x:v>
+        <x:v>Lê Thị Thuý</x:v>
       </x:c>
       <x:c r="E7" s="26" t="str">
-        <x:v>Báo cáo QA; log trích nguồn; log làm lại; feedback ticket</x:v>
+        <x:v>QA report + escalation log + lỗi theo severity</x:v>
       </x:c>
       <x:c r="F7" s="26" t="str">
-        <x:v>Nguồn kiểm chứng ≥95%; rework ≤10%; ≥70% tác vụ phù hợp dùng workflow mới; 0 vi phạm ACL</x:v>
+        <x:v>100% ca phức tạp có đường chuyển; 0 lỗi nghiêm trọng; CSAT index ≥100</x:v>
       </x:c>
       <x:c r="G7" s="26" t="str">
-        <x:v>Sửa retrieval, nguồn, handoff hoặc hướng dẫn; giữ pilot</x:v>
+        <x:v>Giữ pilot; tăng human review; sửa routing</x:v>
       </x:c>
       <x:c r="H7" s="63" t="str">
-        <x:v>CHỜ GATE 30</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="100" customHeight="1">
+        <x:v>ĐANG SỬA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="96" customHeight="1">
       <x:c r="A8" s="26" t="str">
         <x:v>61–90 ngày</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>Quyết định mở rộng / sửa / dừng</x:v>
+        <x:v>Quyết định scale</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>Đối chiếu mục tiêu; kiểm governance; xác nhận owner vận hành; đánh giá lợi ích theo workflow.</x:v>
+        <x:v>Đối chiếu 6 metric; xác nhận owner vận hành; phê duyệt governance và human option.</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>Chủ quy trình (Trần Thị Kiều Oanh)</x:v>
+        <x:v>Trần Thị Kiều Oanh</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>Biên bản gate; dashboard đủ dữ liệu; quyết định ký bởi sponsor</x:v>
+        <x:v>Biên bản gate + dashboard + sponsor sign-off</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>Tất cả metric bắt buộc đạt; thời gian trung vị ≤8 phút; 0 sự cố truy cập nghiêm trọng</x:v>
+        <x:v>Không còn quality-risk flag; năng suất không giảm quá 10%</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>SỬA thêm một vòng hoặc DỪNG theo quy tắc</x:v>
+        <x:v>SỬA thêm một vòng hoặc DỪNG workflow rủi ro</x:v>
       </x:c>
       <x:c r="H8" s="63" t="str">
         <x:v>CHỜ GATE 60</x:v>
@@ -1859,11 +1813,6 @@
     <x:mergeCell ref="A1:H2"/>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H6:H8">
-      <x:formula1>"CHƯA BẮT ĐẦU,ĐANG LÀM,ĐẠT,KHÔNG ĐẠT,CHỜ GATE 30,CHỜ GATE 60"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -1872,21 +1821,22 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="29" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="29" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="42" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="46" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>METRICS — TỪ SỬ DỤNG ĐẾN GIÁ TRỊ</x:v>
+        <x:v>METRICS — BASELINE &amp; KẾT QUẢ CÔNG KHAI</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -1897,6 +1847,7 @@
       <x:c r="H1" s="4"/>
       <x:c r="I1" s="4"/>
       <x:c r="J1" s="4"/>
+      <x:c r="K1" s="4"/>
     </x:row>
     <x:row r="2" ht="15" customHeight="1">
       <x:c r="A2" s="4"/>
@@ -1909,10 +1860,11 @@
       <x:c r="H2" s="4"/>
       <x:c r="I2" s="4"/>
       <x:c r="J2" s="4"/>
-    </x:row>
-    <x:row r="3" ht="34" customHeight="1">
+      <x:c r="K2" s="4"/>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>Nhập kết quả mới nhất ở cột G (màu vàng). Cột I tự đánh giá theo chiều mục tiêu và dẫn tới hành động cụ thể.</x:v>
+        <x:v>Dữ liệu baseline/kết quả lấy từ hồ sơ SEC/Klarna. Trạng thái và quyết định tự tính; không còn ô dữ liệu nháp.</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -1923,13 +1875,14 @@
       <x:c r="H3" s="8"/>
       <x:c r="I3" s="8"/>
       <x:c r="J3" s="8"/>
+      <x:c r="K3" s="8"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="56" t="str">
         <x:v>Tầng</x:v>
       </x:c>
       <x:c r="B5" s="57" t="str">
-        <x:v>Cấp metric</x:v>
+        <x:v>Cấp</x:v>
       </x:c>
       <x:c r="C5" s="57" t="str">
         <x:v>Chỉ số</x:v>
@@ -1944,7 +1897,7 @@
         <x:v>Mục tiêu</x:v>
       </x:c>
       <x:c r="G5" s="57" t="str">
-        <x:v>Kết quả mới nhất</x:v>
+        <x:v>Kết quả</x:v>
       </x:c>
       <x:c r="H5" s="57" t="str">
         <x:v>Nguồn dữ liệu</x:v>
@@ -1952,11 +1905,14 @@
       <x:c r="I5" s="57" t="str">
         <x:v>Trạng thái</x:v>
       </x:c>
-      <x:c r="J5" s="58" t="str">
-        <x:v>Owner / khi chỉ số xấu</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="66" customHeight="1">
+      <x:c r="J5" s="57" t="str">
+        <x:v>Owner / hành động khi xấu</x:v>
+      </x:c>
+      <x:c r="K5" s="58" t="str">
+        <x:v>URL nguồn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="74" customHeight="1">
       <x:c r="A6" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -1964,30 +1920,35 @@
         <x:v>Product</x:v>
       </x:c>
       <x:c r="C6" s="24" t="str">
-        <x:v>Tỷ lệ tác vụ phù hợp dùng workflow AI</x:v>
-      </x:c>
-      <x:c r="D6" s="24" t="str">
-        <x:v>Chưa đo — kế hoạch: tuần 1 pilot</x:v>
+        <x:v>Tỷ lệ chat CSKH do AI xử lý</x:v>
+      </x:c>
+      <x:c r="D6" s="64" t="n">
+        <x:v>0.66</x:v>
       </x:c>
       <x:c r="E6" s="24" t="str">
         <x:v>&gt;=</x:v>
       </x:c>
-      <x:c r="F6" s="70" t="n">
-        <x:v>0.7</x:v>
-      </x:c>
-      <x:c r="G6" s="68"/>
+      <x:c r="F6" s="64" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="G6" s="64" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
       <x:c r="H6" s="24" t="str">
-        <x:v>Log tác vụ + danh mục workflow</x:v>
+        <x:v>Service chat log công bố trong hồ sơ SEC</x:v>
       </x:c>
       <x:c r="I6" s="24" t="str">
-        <x:f>IF(G6="","CHƯA ĐO",IF(E6="&gt;=",IF(G6&gt;=F6,"ĐẠT","XẤU"),IF(G6&lt;=F6,"ĐẠT","XẤU")))</x:f>
-        <x:v>CHƯA ĐO</x:v>
+        <x:f>IF(E6="&gt;=",IF(G6&gt;=F6,"ĐẠT","XẤU"),IF(G6&lt;=F6,"ĐẠT","XẤU"))</x:f>
+        <x:v>ĐẠT</x:v>
       </x:c>
       <x:c r="J6" s="24" t="str">
-        <x:v>AI Product Owner (Giang Minh Phú) — phỏng vấn nhanh, tìm friction theo bước; sửa prompt/UI/handoff.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="66" customHeight="1">
+        <x:v>Giang Minh Phú — nếu giảm: phân tích intent/routing; không ép usage bằng mọi giá.</x:v>
+      </x:c>
+      <x:c r="K6" s="24" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000200329226000007/klar-20251231.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="74" customHeight="1">
       <x:c r="A7" s="26" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -1995,30 +1956,35 @@
         <x:v>Workflow</x:v>
       </x:c>
       <x:c r="C7" s="26" t="str">
-        <x:v>Tỷ lệ mở nguồn trước khi sử dụng kết quả</x:v>
-      </x:c>
-      <x:c r="D7" s="26" t="str">
-        <x:v>Chưa đo — kế hoạch: tuần 1 pilot</x:v>
+        <x:v>Thời gian xử lý trung bình (phút)</x:v>
+      </x:c>
+      <x:c r="D7" s="26" t="n">
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E7" s="26" t="str">
-        <x:v>&gt;=</x:v>
-      </x:c>
-      <x:c r="F7" s="71" t="n">
-        <x:v>0.9</x:v>
-      </x:c>
-      <x:c r="G7" s="69"/>
+        <x:v>&lt;=</x:v>
+      </x:c>
+      <x:c r="F7" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G7" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="H7" s="26" t="str">
-        <x:v>Click log nguồn + task log</x:v>
+        <x:v>Service chat log: human 12 phút, AI 2 phút</x:v>
       </x:c>
       <x:c r="I7" s="26" t="str">
-        <x:f>IF(G7="","CHƯA ĐO",IF(E7="&gt;=",IF(G7&gt;=F7,"ĐẠT","XẤU"),IF(G7&lt;=F7,"ĐẠT","XẤU")))</x:f>
-        <x:v>CHƯA ĐO</x:v>
+        <x:f>IF(E7="&gt;=",IF(G7&gt;=F7,"ĐẠT","XẤU"),IF(G7&lt;=F7,"ĐẠT","XẤU"))</x:f>
+        <x:v>ĐẠT</x:v>
       </x:c>
       <x:c r="J7" s="26" t="str">
-        <x:v>Trưởng nhóm vận hành (Trần Thị Kiều Oanh) — coaching tại bước kiểm chứng; chặn hoàn tất nếu chưa mở nguồn.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="66" customHeight="1">
+        <x:v>Trần Thị Kiều Oanh — nếu tăng: xem lại routing, retrieval và handoff.</x:v>
+      </x:c>
+      <x:c r="K7" s="26" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000200329226000007/klar-20251231.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="74" customHeight="1">
       <x:c r="A8" s="26" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -2026,30 +1992,35 @@
         <x:v>Workflow</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>Thời gian trung vị hoàn thành tra cứu (phút)</x:v>
-      </x:c>
-      <x:c r="D8" s="26" t="str">
-        <x:v>Chưa đo — kế hoạch: tuần 1 pilot</x:v>
+        <x:v>Chỉ số câu hỏi lặp lại (trước AI = 100)</x:v>
+      </x:c>
+      <x:c r="D8" s="26" t="n">
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
         <x:v>&lt;=</x:v>
       </x:c>
       <x:c r="F8" s="26" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="G8" s="69"/>
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="G8" s="26" t="n">
+        <x:v>75</x:v>
+      </x:c>
       <x:c r="H8" s="26" t="str">
-        <x:v>Timestamp task start/end</x:v>
+        <x:v>Repeat inquiries giảm 25% sau launch</x:v>
       </x:c>
       <x:c r="I8" s="26" t="str">
-        <x:f>IF(G8="","CHƯA ĐO",IF(E8="&gt;=",IF(G8&gt;=F8,"ĐẠT","XẤU"),IF(G8&lt;=F8,"ĐẠT","XẤU")))</x:f>
-        <x:v>CHƯA ĐO</x:v>
+        <x:f>IF(E8="&gt;=",IF(G8&gt;=F8,"ĐẠT","XẤU"),IF(G8&lt;=F8,"ĐẠT","XẤU"))</x:f>
+        <x:v>ĐẠT</x:v>
       </x:c>
       <x:c r="J8" s="26" t="str">
-        <x:v>Chủ quy trình (Trần Thị Kiều Oanh) — xem lại bước thừa, retrieval và handoff.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="66" customHeight="1">
+        <x:v>Trần Thị Kiều Oanh — nếu &gt;75: phân loại nguyên nhân và tăng human follow-up.</x:v>
+      </x:c>
+      <x:c r="K8" s="26" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000200329226000007/klar-20251231.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="74" customHeight="1">
       <x:c r="A9" s="26" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -2057,72 +2028,82 @@
         <x:v>Product</x:v>
       </x:c>
       <x:c r="C9" s="26" t="str">
-        <x:v>Tỷ lệ câu trả lời có nguồn và ngày cập nhật</x:v>
-      </x:c>
-      <x:c r="D9" s="26" t="str">
-        <x:v>Chưa đo — kế hoạch: QA mẫu tuần 1</x:v>
+        <x:v>CSAT tương đối (human = 100)</x:v>
+      </x:c>
+      <x:c r="D9" s="26" t="n">
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E9" s="26" t="str">
         <x:v>&gt;=</x:v>
       </x:c>
-      <x:c r="F9" s="71" t="n">
-        <x:v>0.95</x:v>
-      </x:c>
-      <x:c r="G9" s="69"/>
+      <x:c r="F9" s="26" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G9" s="26" t="n">
+        <x:v>100</x:v>
+      </x:c>
       <x:c r="H9" s="26" t="str">
-        <x:v>Log câu trả lời + QA mẫu 10%</x:v>
+        <x:v>Khảo sát nội bộ công bố: AI on-par human</x:v>
       </x:c>
       <x:c r="I9" s="26" t="str">
-        <x:f>IF(G9="","CHƯA ĐO",IF(E9="&gt;=",IF(G9&gt;=F9,"ĐẠT","XẤU"),IF(G9&lt;=F9,"ĐẠT","XẤU")))</x:f>
-        <x:v>CHƯA ĐO</x:v>
+        <x:f>IF(E9="&gt;=",IF(G9&gt;=F9,"ĐẠT","XẤU"),IF(G9&lt;=F9,"ĐẠT","XẤU"))</x:f>
+        <x:v>ĐẠT</x:v>
       </x:c>
       <x:c r="J9" s="26" t="str">
-        <x:v>AI Product Owner (Giang Minh Phú) — tắt nguồn lỗi; sửa retrieval và bắt buộc citation.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="66" customHeight="1">
+        <x:v>Lê Thị Thuý — nếu &lt;100: QA theo phân khúc/intent và tăng human option.</x:v>
+      </x:c>
+      <x:c r="K9" s="26" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000200329226000007/klar-20251231.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="74" customHeight="1">
       <x:c r="A10" s="26" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B10" s="26" t="str">
-        <x:v>Workflow</x:v>
+        <x:v>Value</x:v>
       </x:c>
       <x:c r="C10" s="26" t="str">
-        <x:v>Tỷ lệ hoàn thành không cần QA làm lại</x:v>
-      </x:c>
-      <x:c r="D10" s="26" t="str">
-        <x:v>Chưa đo — kế hoạch: QA mẫu tuần 1</x:v>
+        <x:v>Tiết kiệm chi phí năm/annualized (triệu USD)</x:v>
+      </x:c>
+      <x:c r="D10" s="26" t="n">
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E10" s="26" t="str">
         <x:v>&gt;=</x:v>
       </x:c>
-      <x:c r="F10" s="71" t="n">
-        <x:v>0.9</x:v>
-      </x:c>
-      <x:c r="G10" s="69"/>
+      <x:c r="F10" s="26" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G10" s="26" t="n">
+        <x:v>58</x:v>
+      </x:c>
       <x:c r="H10" s="26" t="str">
-        <x:v>QA checklist + ticket rework</x:v>
+        <x:v>2024: 39m; annualized Sep-2025: 58m</x:v>
       </x:c>
       <x:c r="I10" s="26" t="str">
-        <x:f>IF(G10="","CHƯA ĐO",IF(E10="&gt;=",IF(G10&gt;=F10,"ĐẠT","XẤU"),IF(G10&lt;=F10,"ĐẠT","XẤU")))</x:f>
-        <x:v>CHƯA ĐO</x:v>
+        <x:f>IF(E10="&gt;=",IF(G10&gt;=F10,"ĐẠT","XẤU"),IF(G10&lt;=F10,"ĐẠT","XẤU"))</x:f>
+        <x:v>ĐẠT</x:v>
       </x:c>
       <x:c r="J10" s="26" t="str">
-        <x:v>QA Lead (Lê Thị Thuý) — tăng QA mẫu; phân loại lỗi; sửa checklist / nguồn.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="66" customHeight="1">
+        <x:v>Giang Minh Phú — nếu &lt;40: rà cost-to-serve nhưng không cắt quality control.</x:v>
+      </x:c>
+      <x:c r="K10" s="26" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000162828025052805/exhibit992klarnapresenta.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="74" customHeight="1">
       <x:c r="A11" s="26" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B11" s="26" t="str">
         <x:v>Risk</x:v>
       </x:c>
       <x:c r="C11" s="26" t="str">
-        <x:v>Số sự cố truy cập tài liệu ngoài quyền</x:v>
-      </x:c>
-      <x:c r="D11" s="26" t="str">
-        <x:v>Chưa đo — kế hoạch: audit log tuần 1</x:v>
+        <x:v>Tín hiệu công khai về chất lượng thấp hơn (0/1)</x:v>
+      </x:c>
+      <x:c r="D11" s="26" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E11" s="26" t="str">
         <x:v>&lt;=</x:v>
@@ -2130,21 +2111,26 @@
       <x:c r="F11" s="26" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G11" s="69"/>
+      <x:c r="G11" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="H11" s="26" t="str">
-        <x:v>Security/ACL audit log</x:v>
+        <x:v>SEC staff letter dẫn phát biểu CEO về lower quality</x:v>
       </x:c>
       <x:c r="I11" s="26" t="str">
-        <x:f>IF(G11="","CHƯA ĐO",IF(E11="&gt;=",IF(G11&gt;=F11,"ĐẠT","XẤU"),IF(G11&lt;=F11,"ĐẠT","XẤU")))</x:f>
-        <x:v>CHƯA ĐO</x:v>
+        <x:f>IF(E11="&gt;=",IF(G11&gt;=F11,"ĐẠT","XẤU"),IF(G11&lt;=F11,"ĐẠT","XẤU"))</x:f>
+        <x:v>XẤU</x:v>
       </x:c>
       <x:c r="J11" s="26" t="str">
-        <x:v>Security Owner (Lê Thị Thuý) — dừng pilot liên quan, cô lập nguồn, điều tra và sửa ACL.</x:v>
+        <x:v>Lê Thị Thuý — quality stop: tăng human-in-the-loop, SLA escalation và QA mẫu.</x:v>
+      </x:c>
+      <x:c r="K11" s="26" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2003292/000000000025005760/filename1.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="11" t="str">
-        <x:v>QUY TẮC DỮ LIỆU</x:v>
+        <x:v>GHI CHÚ ĐỊNH NGHĨA</x:v>
       </x:c>
       <x:c r="B13" s="11"/>
       <x:c r="C13" s="11"/>
@@ -2155,13 +2141,14 @@
       <x:c r="H13" s="11"/>
       <x:c r="I13" s="11"/>
       <x:c r="J13" s="11"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="72" t="str">
-        <x:v>Định nghĩa mẫu</x:v>
+      <x:c r="K13" s="11"/>
+    </x:row>
+    <x:row r="14" ht="38" customHeight="1">
+      <x:c r="A14" s="23" t="str">
+        <x:v>CSAT index</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
-        <x:v>Pilot 20–30 nhân viên vận hành; đo theo từng workflow, không gộp câu hỏi ngoài phạm vi.</x:v>
+        <x:v>Do nguồn chỉ công bố 'on-par', quy đổi human=100 và AI=100; không diễn giải thành điểm CSAT tuyệt đối.</x:v>
       </x:c>
       <x:c r="C14" s="24"/>
       <x:c r="D14" s="24"/>
@@ -2171,13 +2158,14 @@
       <x:c r="H14" s="24"/>
       <x:c r="I14" s="24"/>
       <x:c r="J14" s="24"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="73" t="str">
-        <x:v>Chu kỳ cập nhật</x:v>
+      <x:c r="K14" s="24"/>
+    </x:row>
+    <x:row r="15" ht="38" customHeight="1">
+      <x:c r="A15" s="25" t="str">
+        <x:v>Repeat index</x:v>
       </x:c>
       <x:c r="B15" s="26" t="str">
-        <x:v>Hằng tuần trong pilot; QA lấy mẫu ngẫu nhiên tối thiểu 10% tác vụ.</x:v>
+        <x:v>Baseline trước AI=100; giảm 25% tương ứng kết quả=75. Đây là chỉ số chuẩn hoá, không phải số ticket tuyệt đối.</x:v>
       </x:c>
       <x:c r="C15" s="26"/>
       <x:c r="D15" s="26"/>
@@ -2187,13 +2175,14 @@
       <x:c r="H15" s="26"/>
       <x:c r="I15" s="26"/>
       <x:c r="J15" s="26"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="73" t="str">
-        <x:v>Data owner</x:v>
+      <x:c r="K15" s="26"/>
+    </x:row>
+    <x:row r="16" ht="38" customHeight="1">
+      <x:c r="A16" s="25" t="str">
+        <x:v>Quality flag</x:v>
       </x:c>
       <x:c r="B16" s="26" t="str">
-        <x:v>AI Product Owner (Giang Minh Phú) chịu dữ liệu product; Chủ quy trình (Trần Thị Kiều Oanh) chịu metric workflow; QA Lead và Security Owner (Lê Thị Thuý) chịu metric chất lượng và rủi ro.</x:v>
+        <x:v>Biến nhị phân dựa trên bằng chứng công khai: 1 khi có tín hiệu lower quality cần quality gate; target=0.</x:v>
       </x:c>
       <x:c r="C16" s="26"/>
       <x:c r="D16" s="26"/>
@@ -2203,37 +2192,20 @@
       <x:c r="H16" s="26"/>
       <x:c r="I16" s="26"/>
       <x:c r="J16" s="26"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="73" t="str">
-        <x:v>Tình trạng dữ liệu</x:v>
-      </x:c>
-      <x:c r="B17" s="26" t="str">
-        <x:v>Tại thời điểm nộp chưa có kết quả pilot thật. Cột Baseline và Kết quả để trống có chủ ý — không điền số giả; trạng thái tự tính là CHƯA ĐO cho cả 6 chỉ số.</x:v>
-      </x:c>
-      <x:c r="C17" s="26"/>
-      <x:c r="D17" s="26"/>
-      <x:c r="E17" s="26"/>
-      <x:c r="F17" s="26"/>
-      <x:c r="G17" s="26"/>
-      <x:c r="H17" s="26"/>
-      <x:c r="I17" s="26"/>
-      <x:c r="J17" s="26"/>
+      <x:c r="K16" s="26"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J2"/>
-    <x:mergeCell ref="A3:J3"/>
-    <x:mergeCell ref="A13:J13"/>
-    <x:mergeCell ref="B14:J14"/>
-    <x:mergeCell ref="B15:J15"/>
-    <x:mergeCell ref="B16:J16"/>
-    <x:mergeCell ref="B17:J17"/>
+    <x:mergeCell ref="A1:K2"/>
+    <x:mergeCell ref="A3:K3"/>
+    <x:mergeCell ref="A13:K13"/>
+    <x:mergeCell ref="B14:K14"/>
+    <x:mergeCell ref="B15:K15"/>
+    <x:mergeCell ref="B16:K16"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="I6:I11">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="ĐẠT"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="XẤU"/>
-    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="CHƯA ĐO"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2245,11 +2217,11 @@
   <x:cols>
     <x:col min="1" max="1" width="7" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -2275,9 +2247,9 @@
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
     </x:row>
-    <x:row r="3" ht="34" customHeight="1">
+    <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>Ghi nhận góp ý cụ thể và dấu vết chỉnh sửa để chứng minh v2 khác v1.</x:v>
+        <x:v>Nhóm phản biện: Flaiiin | Ba thay đổi có thể đối chiếu trực tiếp giữa v1 và v2.</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -2292,10 +2264,10 @@
         <x:v>#</x:v>
       </x:c>
       <x:c r="B5" s="57" t="str">
-        <x:v>Trục phản biện</x:v>
+        <x:v>Trục</x:v>
       </x:c>
       <x:c r="C5" s="57" t="str">
-        <x:v>Góp ý nhóm bạn</x:v>
+        <x:v>Góp ý nhận từ Flaiiin</x:v>
       </x:c>
       <x:c r="D5" s="57" t="str">
         <x:v>Vấn đề ở v1</x:v>
@@ -2304,7 +2276,7 @@
         <x:v>Thay đổi trong v2</x:v>
       </x:c>
       <x:c r="F5" s="57" t="str">
-        <x:v>Sheet / vị trí</x:v>
+        <x:v>Vị trí</x:v>
       </x:c>
       <x:c r="G5" s="57" t="str">
         <x:v>Owner</x:v>
@@ -2313,7 +2285,7 @@
         <x:v>Trạng thái</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="82" customHeight="1">
+    <x:row r="6" ht="78" customHeight="1">
       <x:c r="A6" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -2321,51 +2293,51 @@
         <x:v>Chỉ số</x:v>
       </x:c>
       <x:c r="C6" s="24" t="str">
-        <x:v>Số login và số câu hỏi chỉ là activity, chưa chứng minh giá trị.</x:v>
+        <x:v>Activity/volume chưa chứng minh adoption có chất lượng.</x:v>
       </x:c>
       <x:c r="D6" s="24" t="str">
-        <x:v>Metric thiên về usage; thiếu workflow quality.</x:v>
+        <x:v>V1 nhấn volume và cost; chưa có quality gate.</x:v>
       </x:c>
       <x:c r="E6" s="24" t="str">
-        <x:v>Thêm tỷ lệ mở nguồn, thời gian từ log, tỷ lệ không cần QA làm lại và sự cố ACL.</x:v>
+        <x:v>Thêm CSAT index, repeat inquiry, quality-risk flag và action khi xấu.</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
-        <x:v>Metrics!A5:J11</x:v>
+        <x:v>Metrics!A5:K16</x:v>
       </x:c>
       <x:c r="G6" s="24" t="str">
-        <x:v>AI Product Owner (Giang Minh Phú)</x:v>
+        <x:v>Giang Minh Phú</x:v>
       </x:c>
       <x:c r="H6" s="24" t="str">
         <x:v>ĐÃ SỬA</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="82" customHeight="1">
+    <x:row r="7" ht="78" customHeight="1">
       <x:c r="A7" s="26" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B7" s="26" t="str">
-        <x:v>Hành động</x:v>
+        <x:v>Workflow</x:v>
       </x:c>
       <x:c r="C7" s="26" t="str">
-        <x:v>Chưa rõ ai chịu trách nhiệm và xử lý khi AI không chắc.</x:v>
+        <x:v>Chưa rõ quyền cuối và cách xử lý ca phức tạp.</x:v>
       </x:c>
       <x:c r="D7" s="26" t="str">
-        <x:v>TO-BE chỉ có bước hỏi AI; chưa có handoff/RACI.</x:v>
+        <x:v>Handoff chỉ ghi chung là chuyển người.</x:v>
       </x:c>
       <x:c r="E7" s="26" t="str">
-        <x:v>Thêm người phê duyệt cuối, SME escalation, ticket phản hồi và owner từng bước.</x:v>
+        <x:v>Thêm taxonomy, confidence gate, SLA chuyển người và RACI.</x:v>
       </x:c>
       <x:c r="F7" s="26" t="str">
         <x:v>Workflow!F6:I18</x:v>
       </x:c>
       <x:c r="G7" s="26" t="str">
-        <x:v>Chủ quy trình (Trần Thị Kiều Oanh)</x:v>
+        <x:v>Trần Thị Kiều Oanh</x:v>
       </x:c>
       <x:c r="H7" s="26" t="str">
         <x:v>ĐÃ SỬA</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="82" customHeight="1">
+    <x:row r="8" ht="78" customHeight="1">
       <x:c r="A8" s="26" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -2373,19 +2345,19 @@
         <x:v>Roadmap</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>30–60–90 là danh sách việc, chưa có gate.</x:v>
+        <x:v>30–60–90 chưa phải cổng quyết định.</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>Không có tiêu chí qua giai đoạn.</x:v>
+        <x:v>Thiếu tiêu chí qua cổng và phương án fail.</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>Thêm bằng chứng, tiêu chí qua cổng và hành động nếu không đạt cho từng giai đoạn.</x:v>
+        <x:v>Thêm evidence, gate criteria và hành động nếu không đạt.</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
         <x:v>Roadmap 30-60-90!A5:H8</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Sponsor</x:v>
+        <x:v>Lê Thị Thuý</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str">
         <x:v>ĐÃ SỬA</x:v>
@@ -2403,12 +2375,12 @@
       <x:c r="G10" s="11"/>
       <x:c r="H10" s="11"/>
     </x:row>
-    <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="74" t="str">
+    <x:row r="11" ht="44" customHeight="1">
+      <x:c r="A11" s="70" t="str">
         <x:v>Quyết định</x:v>
       </x:c>
       <x:c r="B11" s="24" t="str">
-        <x:v>SỬA — tiếp tục pilot có điều kiện, chưa rollout rộng</x:v>
+        <x:v>SỬA — tiếp tục AI cho ca thường, tăng human-in-the-loop cho ca phức tạp</x:v>
       </x:c>
       <x:c r="C11" s="24"/>
       <x:c r="D11" s="24"/>
@@ -2417,12 +2389,12 @@
       <x:c r="G11" s="24"/>
       <x:c r="H11" s="24"/>
     </x:row>
-    <x:row r="12" ht="42" customHeight="1">
-      <x:c r="A12" s="75" t="str">
+    <x:row r="12" ht="44" customHeight="1">
+      <x:c r="A12" s="71" t="str">
         <x:v>Lý do</x:v>
       </x:c>
       <x:c r="B12" s="26" t="str">
-        <x:v>Hai nguyên nhân gốc là workflow chưa chính thức và thiếu kiến trúc tin cậy; cả hai có thể sửa trong pilot và đo được.</x:v>
+        <x:v>5/6 metric đạt nhưng quality-risk flag xấu; usage và cost không được lấn át chất lượng.</x:v>
       </x:c>
       <x:c r="C12" s="26"/>
       <x:c r="D12" s="26"/>
@@ -2431,12 +2403,12 @@
       <x:c r="G12" s="26"/>
       <x:c r="H12" s="26"/>
     </x:row>
-    <x:row r="13" ht="42" customHeight="1">
-      <x:c r="A13" s="75" t="str">
+    <x:row r="13" ht="44" customHeight="1">
+      <x:c r="A13" s="71" t="str">
         <x:v>Bước tiếp theo</x:v>
       </x:c>
       <x:c r="B13" s="26" t="str">
-        <x:v>Trong 30 ngày: khoá nguồn, ACL, owner; đo baseline; triển khai TO-BE cho 20–30 người vận hành.</x:v>
+        <x:v>Chuẩn hoá taxonomy, SLA chuyển người, QA mẫu phân tầng; chỉ scale khi quality flag về 0.</x:v>
       </x:c>
       <x:c r="C13" s="26"/>
       <x:c r="D13" s="26"/>

</xml_diff>